<commit_message>
Update runtime assets and manifest metadata
</commit_message>
<xml_diff>
--- a/assets_cropped/Tsurumaru Tsuyoshi/manifest_edit.xlsx
+++ b/assets_cropped/Tsurumaru Tsuyoshi/manifest_edit.xlsx
@@ -5,22 +5,23 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\TanukiProject\venv\assets_cropped\Tsurumaru Tsuyoshi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\TanukiProject\tanuki_app\assets_cropped\Tsurumaru Tsuyoshi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0118E261-8101-45B2-B24B-B5E78EDA9256}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1776A0-449F-44BE-AD86-B9498FCCF5B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18510" windowHeight="5625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="stale_backup" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="200">
   <si>
     <t>filename</t>
   </si>
@@ -40,356 +41,631 @@
     <t>drag_fly-angry.gif</t>
   </si>
   <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>drag_fly-cry.gif</t>
+  </si>
+  <si>
+    <t>drag_fly-happy.gif</t>
+  </si>
+  <si>
+    <t>normal</t>
+  </si>
+  <si>
+    <t>drag_fly-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>drag_fly-laugh.gif</t>
+  </si>
+  <si>
+    <t>drag_fly-sad.gif</t>
+  </si>
+  <si>
+    <t>drag_fly-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_drink-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_drink-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_drink-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_eat-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_eat-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_eat-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_eat-think.gif</t>
+  </si>
+  <si>
+    <t>idle_get-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_get-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_get-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_get-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_get-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_get-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-exhausted.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-sleep.gif</t>
+  </si>
+  <si>
+    <t>idle_lie-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_rest-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_rest-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_rest-mad.gif</t>
+  </si>
+  <si>
+    <t>idle_rest-sleep.gif</t>
+  </si>
+  <si>
+    <t>idle_rest-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side-scared.gif</t>
+  </si>
+  <si>
+    <t>idle_side-sleep.gif</t>
+  </si>
+  <si>
+    <t>idle_side-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side-think.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hand-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hand-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_stretch-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_stretch-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_fan-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_hug-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_hug-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_hug-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_hug-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_hug-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side_hug-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_ready-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_ready-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_rub-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_rub-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_rub-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side_rub-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-hard-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side_shake-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stand-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stand-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stand-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stand-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stand_cheer-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stand_cheer-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stretch-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stretch-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stretch-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stretch-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stretch-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side_stretch-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_no-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_no-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_no-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_no-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_no-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_no-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_squat-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_squat-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_squat-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_squat-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_squat-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_squat-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_stand-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_stand-sad.gif</t>
+  </si>
+  <si>
+    <t>move_climb-angry.gif</t>
+  </si>
+  <si>
+    <t>move_climb-cry.gif</t>
+  </si>
+  <si>
+    <t>move_climb-happy.gif</t>
+  </si>
+  <si>
+    <t>move_climb-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>move_climb-sad.gif</t>
+  </si>
+  <si>
+    <t>move_climb-smile.gif</t>
+  </si>
+  <si>
+    <t>move_fly-angry.gif</t>
+  </si>
+  <si>
+    <t>move_fly-happy.gif</t>
+  </si>
+  <si>
+    <t>move_fly-sad.gif</t>
+  </si>
+  <si>
+    <t>move_fly-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hug-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hug-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hug-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hug-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_hug-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_side_face_stretch-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_sulking-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_side_sulking-think.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_hug-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_hug-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_hug-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_stretch-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_stretch-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_stretch-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_stretch-hard-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave_stretch-mad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-hard-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-hard-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-mad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_wave-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-cry.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-mad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-smile.gif</t>
+  </si>
+  <si>
+    <t>backup_original_filename</t>
+  </si>
+  <si>
+    <t>backup_character</t>
+  </si>
+  <si>
+    <t>backup_reason</t>
+  </si>
+  <si>
+    <t>idle_side_face_stretch-happy.gif__Tsurumaru Tsuyoshi</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Tsurumaru Tsuyoshi</t>
+  </si>
+  <si>
+    <t>stale_filename_not_found</t>
+  </si>
+  <si>
+    <t>idle_side_face_stretch-smile.gif__Tsurumaru Tsuyoshi</t>
+  </si>
+  <si>
     <t>low</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>move_fly-cry.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>move_fly-hard-cry.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>move_fly-laugh.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>idle_side_music-smile.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>future_work</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>side_ready_followup</t>
+  </si>
+  <si>
+    <t>side_ready_followup</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_child_comfort</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_preview</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>drag</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>care_child_comfort,offer_accept_milk,bottle_feed_child_drink</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>drag,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>care_child_comfort,offer_accept_milk,bottle_feed_child_drink,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_preview,offer_denied,offer_timeout_route_a_step1,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_preview,offer_denied,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_preview,offer_denied,offer_timeout_route_b_step1,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_denied,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_child_comfort,offer_denied,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_child_comfort,offer_timeout_route_a_step2,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_child_comfort,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>side_ready_followup,negative_reaction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>negative_reaction,hard_landing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>random</t>
-  </si>
-  <si>
-    <t>drag_fly-cry.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_denied,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_denied,negative_reaction,hard_landing,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,relation_watch,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,post_observe,offer_denied,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,post_observe,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,post_observe,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,relation_watch,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,offer_timeout_route_a_step3,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,bottle_feed_child_approach,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,bottle_feed_child_approach,negative_reaction,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,random</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>severe</t>
-  </si>
-  <si>
-    <t>drag_fly-happy.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>normal</t>
-  </si>
-  <si>
-    <t>drag_fly-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>drag_fly-laugh.gif</t>
-  </si>
-  <si>
-    <t>drag_fly-sad.gif</t>
-  </si>
-  <si>
-    <t>drag_fly-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_drink-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_drink-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_drink-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_eat-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_eat-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_eat-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_eat-think.gif</t>
-  </si>
-  <si>
-    <t>idle_get-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_get-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_get-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_get-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_get-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_get-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-exhausted.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-sleep.gif</t>
-  </si>
-  <si>
-    <t>idle_lie-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_rest-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_rest-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_rest-mad.gif</t>
-  </si>
-  <si>
-    <t>idle_rest-sleep.gif</t>
-  </si>
-  <si>
-    <t>idle_rest-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_side-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_side-scared.gif</t>
-  </si>
-  <si>
-    <t>idle_side-sleep.gif</t>
-  </si>
-  <si>
-    <t>idle_side-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side-think.gif</t>
-  </si>
-  <si>
-    <t>idle_side_face-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_face-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_face_hand-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_face_hand-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_face_stretch-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_face_stretch-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_fan-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_hug-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_hug-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_hug-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_hug-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_hug-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_side_hug-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_play-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_ready-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_ready-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_rub-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_rub-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_rub-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_side_rub-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-hard-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_side_shake-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stand-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stand-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stand-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stand-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stand_cheer-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stand_cheer-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stretch-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stretch-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stretch-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stretch-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stretch-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_side_stretch-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_no-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_no-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_no-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_no-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_no-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_no-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_squat-angry.gif</t>
-  </si>
-  <si>
-    <t>idle_squat-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_squat-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_squat-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>idle_squat-sad.gif</t>
-  </si>
-  <si>
-    <t>idle_squat-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_stand-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_stand-sad.gif</t>
-  </si>
-  <si>
-    <t>move_climb-angry.gif</t>
-  </si>
-  <si>
-    <t>move_climb-cry.gif</t>
-  </si>
-  <si>
-    <t>move_climb-happy.gif</t>
-  </si>
-  <si>
-    <t>move_climb-hard-cry.gif</t>
-  </si>
-  <si>
-    <t>move_climb-sad.gif</t>
-  </si>
-  <si>
-    <t>move_climb-smile.gif</t>
-  </si>
-  <si>
-    <t>move_fly-angry.gif</t>
-  </si>
-  <si>
-    <t>move_fly-happy.gif</t>
-  </si>
-  <si>
-    <t>move_fly-sad.gif</t>
-  </si>
-  <si>
-    <t>move_fly-smile.gif</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>low,severe</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>normal</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>random,drink</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>random,eat</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>random,get</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>low</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>random,lie</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>normal,low</t>
+    <t>normal,low,severe</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,observe_hold,random</t>
+  </si>
+  <si>
+    <t>window_perch,observe_hold</t>
+  </si>
+  <si>
+    <t>window_perch,observe_hold,negative_reaction,random</t>
+  </si>
+  <si>
+    <t>window_perch,observe_hold,offer_timeout_route_b_step2,negative_reaction,random</t>
+  </si>
+  <si>
+    <t>relation_close</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>negative_reaction,relation_close</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,negative_reaction,random,bottle_feed_child_approach</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -762,12 +1038,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
-    <col min="3" max="3" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -792,10 +1068,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>161</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -803,13 +1079,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>113</v>
+        <v>189</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>161</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -817,13 +1093,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>159</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -831,13 +1107,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>189</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>162</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -845,13 +1121,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>190</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>159</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -859,13 +1135,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>161</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -873,13 +1149,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>159</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -887,13 +1163,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -901,13 +1177,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>118</v>
+        <v>191</v>
       </c>
       <c r="C10" t="s">
-        <v>115</v>
+        <v>163</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -915,13 +1191,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -929,13 +1205,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>173</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -943,13 +1219,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>174</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -957,13 +1233,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>6</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -971,13 +1247,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>192</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
+        <v>154</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -985,13 +1261,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="C16" t="s">
-        <v>117</v>
+        <v>164</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -999,13 +1275,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>113</v>
+        <v>189</v>
       </c>
       <c r="C17" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1013,13 +1289,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C18" t="s">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1027,13 +1303,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>189</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1041,13 +1317,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>166</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1055,13 +1331,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1069,13 +1345,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>113</v>
+        <v>189</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>175</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1083,13 +1359,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>192</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1097,13 +1373,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C24" t="s">
-        <v>119</v>
+        <v>173</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1111,13 +1387,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>9</v>
+        <v>189</v>
       </c>
       <c r="C25" t="s">
-        <v>119</v>
+        <v>176</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1125,13 +1401,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C26" t="s">
-        <v>119</v>
+        <v>175</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1139,13 +1415,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>120</v>
+        <v>192</v>
       </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1153,13 +1429,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C28" t="s">
-        <v>119</v>
+        <v>173</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1167,13 +1443,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C29" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1181,13 +1457,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C30" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1195,13 +1471,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="C31" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1209,13 +1485,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>120</v>
+        <v>192</v>
       </c>
       <c r="C32" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -1223,13 +1499,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C33" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -1237,13 +1513,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B34" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C34" t="s">
-        <v>7</v>
+        <v>177</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -1251,13 +1527,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="B35" t="s">
-        <v>113</v>
+        <v>190</v>
       </c>
       <c r="C35" t="s">
-        <v>7</v>
+        <v>177</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -1265,13 +1541,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="B36" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C36" t="s">
-        <v>7</v>
+        <v>178</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -1279,13 +1555,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="B37" t="s">
-        <v>9</v>
+        <v>190</v>
       </c>
       <c r="C37" t="s">
-        <v>7</v>
+        <v>179</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1293,13 +1569,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>45</v>
+        <v>112</v>
       </c>
       <c r="B38" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="C38" t="s">
-        <v>7</v>
+        <v>178</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1307,13 +1583,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>46</v>
+        <v>113</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>149</v>
       </c>
       <c r="C39" t="s">
-        <v>7</v>
+        <v>178</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1321,13 +1597,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>47</v>
+        <v>114</v>
       </c>
       <c r="B40" t="s">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C40" t="s">
-        <v>7</v>
+        <v>179</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1335,13 +1611,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>48</v>
+        <v>115</v>
       </c>
       <c r="B41" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C41" t="s">
-        <v>7</v>
+        <v>180</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1349,13 +1625,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>114</v>
+        <v>190</v>
       </c>
       <c r="C42" t="s">
-        <v>7</v>
+        <v>193</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1363,13 +1639,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C43" t="s">
-        <v>7</v>
+        <v>193</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1377,13 +1653,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C44" t="s">
-        <v>7</v>
+        <v>194</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1391,13 +1667,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C45" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -1405,13 +1681,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C46" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -1419,13 +1695,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C47" t="s">
-        <v>7</v>
+        <v>157</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -1433,13 +1709,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C48" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -1447,13 +1723,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C49" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -1461,13 +1737,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C50" t="s">
-        <v>7</v>
+        <v>157</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -1475,13 +1751,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>58</v>
+        <v>153</v>
       </c>
       <c r="B51" t="s">
-        <v>113</v>
+        <v>190</v>
       </c>
       <c r="C51" t="s">
-        <v>7</v>
+        <v>181</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -1489,13 +1765,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C52" t="s">
-        <v>7</v>
+        <v>182</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -1503,13 +1779,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>9</v>
+        <v>190</v>
       </c>
       <c r="C53" t="s">
-        <v>7</v>
+        <v>181</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -1517,13 +1793,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="C54" t="s">
-        <v>7</v>
+        <v>178</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -1531,13 +1807,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C55" t="s">
-        <v>7</v>
+        <v>179</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -1545,13 +1821,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C56" t="s">
-        <v>7</v>
+        <v>180</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -1559,13 +1835,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C57" t="s">
-        <v>7</v>
+        <v>179</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -1573,13 +1849,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C58" t="s">
-        <v>7</v>
+        <v>169</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -1587,13 +1863,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>118</v>
+        <v>189</v>
       </c>
       <c r="C59" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="D59">
         <v>1</v>
@@ -1601,13 +1877,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C60" t="s">
-        <v>7</v>
+        <v>157</v>
       </c>
       <c r="D60">
         <v>1</v>
@@ -1615,13 +1891,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="C61" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -1629,13 +1905,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C62" t="s">
-        <v>7</v>
+        <v>157</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -1643,13 +1919,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B63" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="C63" t="s">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="D63">
         <v>1</v>
@@ -1657,13 +1933,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
+        <v>190</v>
       </c>
       <c r="C64" t="s">
-        <v>7</v>
+        <v>157</v>
       </c>
       <c r="D64">
         <v>1</v>
@@ -1671,13 +1947,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B65" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C65" t="s">
-        <v>7</v>
+        <v>156</v>
       </c>
       <c r="D65">
         <v>1</v>
@@ -1685,13 +1961,13 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B66" t="s">
-        <v>9</v>
+        <v>190</v>
       </c>
       <c r="C66" t="s">
-        <v>7</v>
+        <v>156</v>
       </c>
       <c r="D66">
         <v>1</v>
@@ -1702,10 +1978,10 @@
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C67" t="s">
-        <v>7</v>
+        <v>171</v>
       </c>
       <c r="D67">
         <v>1</v>
@@ -1716,10 +1992,10 @@
         <v>75</v>
       </c>
       <c r="B68" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="C68" t="s">
-        <v>7</v>
+        <v>171</v>
       </c>
       <c r="D68">
         <v>1</v>
@@ -1730,10 +2006,10 @@
         <v>76</v>
       </c>
       <c r="B69" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C69" t="s">
-        <v>7</v>
+        <v>155</v>
       </c>
       <c r="D69">
         <v>1</v>
@@ -1744,10 +2020,10 @@
         <v>77</v>
       </c>
       <c r="B70" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C70" t="s">
-        <v>7</v>
+        <v>171</v>
       </c>
       <c r="D70">
         <v>1</v>
@@ -1755,13 +2031,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B71" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="C71" t="s">
-        <v>7</v>
+        <v>195</v>
       </c>
       <c r="D71">
         <v>1</v>
@@ -1769,13 +2045,13 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C72" t="s">
-        <v>7</v>
+        <v>196</v>
       </c>
       <c r="D72">
         <v>1</v>
@@ -1783,13 +2059,13 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B73" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C73" t="s">
-        <v>7</v>
+        <v>193</v>
       </c>
       <c r="D73">
         <v>1</v>
@@ -1797,13 +2073,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B74" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C74" t="s">
-        <v>7</v>
+        <v>195</v>
       </c>
       <c r="D74">
         <v>1</v>
@@ -1811,13 +2087,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B75" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C75" t="s">
-        <v>7</v>
+        <v>195</v>
       </c>
       <c r="D75">
         <v>1</v>
@@ -1825,13 +2101,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B76" t="s">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C76" t="s">
-        <v>7</v>
+        <v>193</v>
       </c>
       <c r="D76">
         <v>1</v>
@@ -1839,13 +2115,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="B77" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="C77" t="s">
-        <v>7</v>
+        <v>167</v>
       </c>
       <c r="D77">
         <v>1</v>
@@ -1853,13 +2129,13 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="B78" t="s">
-        <v>11</v>
+        <v>192</v>
       </c>
       <c r="C78" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D78">
         <v>1</v>
@@ -1867,13 +2143,13 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="B79" t="s">
-        <v>9</v>
+        <v>149</v>
       </c>
       <c r="C79" t="s">
-        <v>7</v>
+        <v>183</v>
       </c>
       <c r="D79">
         <v>1</v>
@@ -1881,13 +2157,13 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="B80" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="C80" t="s">
-        <v>7</v>
+        <v>183</v>
       </c>
       <c r="D80">
         <v>1</v>
@@ -1895,13 +2171,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="B81" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C81" t="s">
-        <v>7</v>
+        <v>177</v>
       </c>
       <c r="D81">
         <v>1</v>
@@ -1909,13 +2185,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="B82" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="C82" t="s">
-        <v>7</v>
+        <v>183</v>
       </c>
       <c r="D82">
         <v>1</v>
@@ -1923,13 +2199,13 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="B83" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="C83" t="s">
-        <v>7</v>
+        <v>183</v>
       </c>
       <c r="D83">
         <v>1</v>
@@ -1937,13 +2213,13 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="B84" t="s">
-        <v>11</v>
+        <v>191</v>
       </c>
       <c r="C84" t="s">
-        <v>7</v>
+        <v>183</v>
       </c>
       <c r="D84">
         <v>1</v>
@@ -1951,13 +2227,13 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="B85" t="s">
-        <v>9</v>
+        <v>192</v>
       </c>
       <c r="C85" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D85">
         <v>1</v>
@@ -1965,13 +2241,13 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="B86" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C86" t="s">
-        <v>7</v>
+        <v>177</v>
       </c>
       <c r="D86">
         <v>1</v>
@@ -1979,13 +2255,13 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="B87" t="s">
-        <v>11</v>
+        <v>192</v>
       </c>
       <c r="C87" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D87">
         <v>1</v>
@@ -1993,13 +2269,13 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="C88" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D88">
         <v>1</v>
@@ -2007,13 +2283,13 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>113</v>
+        <v>189</v>
       </c>
       <c r="C89" t="s">
-        <v>7</v>
+        <v>175</v>
       </c>
       <c r="D89">
         <v>1</v>
@@ -2021,13 +2297,13 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C90" t="s">
-        <v>7</v>
+        <v>173</v>
       </c>
       <c r="D90">
         <v>1</v>
@@ -2035,13 +2311,13 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>9</v>
+        <v>189</v>
       </c>
       <c r="C91" t="s">
-        <v>7</v>
+        <v>175</v>
       </c>
       <c r="D91">
         <v>1</v>
@@ -2049,13 +2325,13 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C92" t="s">
-        <v>7</v>
+        <v>175</v>
       </c>
       <c r="D92">
         <v>1</v>
@@ -2063,13 +2339,13 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C93" t="s">
-        <v>7</v>
+        <v>173</v>
       </c>
       <c r="D93">
         <v>1</v>
@@ -2077,13 +2353,13 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="B94" t="s">
-        <v>11</v>
+        <v>190</v>
       </c>
       <c r="C94" t="s">
-        <v>7</v>
+        <v>197</v>
       </c>
       <c r="D94">
         <v>1</v>
@@ -2091,13 +2367,13 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="B95" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C95" t="s">
-        <v>7</v>
+        <v>198</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -2105,13 +2381,13 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="B96" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C96" t="s">
-        <v>7</v>
+        <v>197</v>
       </c>
       <c r="D96">
         <v>1</v>
@@ -2119,13 +2395,13 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="B97" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="C97" t="s">
-        <v>7</v>
+        <v>198</v>
       </c>
       <c r="D97">
         <v>1</v>
@@ -2133,13 +2409,13 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="B98" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C98" t="s">
-        <v>7</v>
+        <v>198</v>
       </c>
       <c r="D98">
         <v>1</v>
@@ -2147,13 +2423,13 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B99" t="s">
-        <v>9</v>
+        <v>189</v>
       </c>
       <c r="C99" t="s">
-        <v>7</v>
+        <v>198</v>
       </c>
       <c r="D99">
         <v>1</v>
@@ -2161,13 +2437,13 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B100" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C100" t="s">
-        <v>7</v>
+        <v>197</v>
       </c>
       <c r="D100">
         <v>1</v>
@@ -2175,13 +2451,13 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="B101" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="C101" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D101">
         <v>1</v>
@@ -2189,13 +2465,13 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="B102" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
       <c r="C102" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D102">
         <v>1</v>
@@ -2203,13 +2479,13 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="B103" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C103" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D103">
         <v>1</v>
@@ -2217,13 +2493,13 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B104" t="s">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="C104" t="s">
-        <v>7</v>
+        <v>173</v>
       </c>
       <c r="D104">
         <v>1</v>
@@ -2231,21 +2507,547 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="B105" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C105" t="s">
-        <v>7</v>
+        <v>174</v>
       </c>
       <c r="D105">
         <v>1</v>
       </c>
     </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>130</v>
+      </c>
+      <c r="B106" t="s">
+        <v>190</v>
+      </c>
+      <c r="C106" t="s">
+        <v>173</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>131</v>
+      </c>
+      <c r="B107" t="s">
+        <v>149</v>
+      </c>
+      <c r="C107" t="s">
+        <v>154</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>132</v>
+      </c>
+      <c r="B108" t="s">
+        <v>149</v>
+      </c>
+      <c r="C108" t="s">
+        <v>174</v>
+      </c>
+      <c r="D108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>133</v>
+      </c>
+      <c r="B109" t="s">
+        <v>190</v>
+      </c>
+      <c r="C109" t="s">
+        <v>173</v>
+      </c>
+      <c r="D109">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>134</v>
+      </c>
+      <c r="B110" t="s">
+        <v>149</v>
+      </c>
+      <c r="C110" t="s">
+        <v>182</v>
+      </c>
+      <c r="D110">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>135</v>
+      </c>
+      <c r="B111" t="s">
+        <v>189</v>
+      </c>
+      <c r="C111" t="s">
+        <v>182</v>
+      </c>
+      <c r="D111">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>136</v>
+      </c>
+      <c r="B112" t="s">
+        <v>190</v>
+      </c>
+      <c r="C112" t="s">
+        <v>181</v>
+      </c>
+      <c r="D112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>137</v>
+      </c>
+      <c r="B113" t="s">
+        <v>149</v>
+      </c>
+      <c r="C113" t="s">
+        <v>181</v>
+      </c>
+      <c r="D113">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>138</v>
+      </c>
+      <c r="B114" t="s">
+        <v>149</v>
+      </c>
+      <c r="C114" t="s">
+        <v>181</v>
+      </c>
+      <c r="D114">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>139</v>
+      </c>
+      <c r="B115" t="s">
+        <v>190</v>
+      </c>
+      <c r="C115" t="s">
+        <v>181</v>
+      </c>
+      <c r="D115">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>92</v>
+      </c>
+      <c r="B116" t="s">
+        <v>149</v>
+      </c>
+      <c r="C116" t="s">
+        <v>182</v>
+      </c>
+      <c r="D116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>93</v>
+      </c>
+      <c r="B117" t="s">
+        <v>189</v>
+      </c>
+      <c r="C117" t="s">
+        <v>182</v>
+      </c>
+      <c r="D117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>94</v>
+      </c>
+      <c r="B118" t="s">
+        <v>190</v>
+      </c>
+      <c r="C118" t="s">
+        <v>181</v>
+      </c>
+      <c r="D118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>95</v>
+      </c>
+      <c r="B119" t="s">
+        <v>189</v>
+      </c>
+      <c r="C119" t="s">
+        <v>182</v>
+      </c>
+      <c r="D119">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>96</v>
+      </c>
+      <c r="B120" t="s">
+        <v>149</v>
+      </c>
+      <c r="C120" t="s">
+        <v>182</v>
+      </c>
+      <c r="D120">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>97</v>
+      </c>
+      <c r="B121" t="s">
+        <v>190</v>
+      </c>
+      <c r="C121" t="s">
+        <v>181</v>
+      </c>
+      <c r="D121">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>98</v>
+      </c>
+      <c r="B122" t="s">
+        <v>190</v>
+      </c>
+      <c r="C122" t="s">
+        <v>181</v>
+      </c>
+      <c r="D122">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>99</v>
+      </c>
+      <c r="B123" t="s">
+        <v>149</v>
+      </c>
+      <c r="C123" t="s">
+        <v>182</v>
+      </c>
+      <c r="D123">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>100</v>
+      </c>
+      <c r="B124" t="s">
+        <v>149</v>
+      </c>
+      <c r="C124" t="s">
+        <v>184</v>
+      </c>
+      <c r="D124">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>101</v>
+      </c>
+      <c r="B125" t="s">
+        <v>189</v>
+      </c>
+      <c r="C125" t="s">
+        <v>185</v>
+      </c>
+      <c r="D125">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>102</v>
+      </c>
+      <c r="B126" t="s">
+        <v>190</v>
+      </c>
+      <c r="C126" t="s">
+        <v>186</v>
+      </c>
+      <c r="D126">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>103</v>
+      </c>
+      <c r="B127" t="s">
+        <v>189</v>
+      </c>
+      <c r="C127" t="s">
+        <v>199</v>
+      </c>
+      <c r="D127">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>104</v>
+      </c>
+      <c r="B128" t="s">
+        <v>149</v>
+      </c>
+      <c r="C128" t="s">
+        <v>187</v>
+      </c>
+      <c r="D128">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>105</v>
+      </c>
+      <c r="B129" t="s">
+        <v>190</v>
+      </c>
+      <c r="C129" t="s">
+        <v>186</v>
+      </c>
+      <c r="D129">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>106</v>
+      </c>
+      <c r="B130" t="s">
+        <v>149</v>
+      </c>
+      <c r="C130" t="s">
+        <v>185</v>
+      </c>
+      <c r="D130">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>150</v>
+      </c>
+      <c r="B131" t="s">
+        <v>189</v>
+      </c>
+      <c r="C131" t="s">
+        <v>185</v>
+      </c>
+      <c r="D131">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>107</v>
+      </c>
+      <c r="B132" t="s">
+        <v>190</v>
+      </c>
+      <c r="C132" t="s">
+        <v>188</v>
+      </c>
+      <c r="D132">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>151</v>
+      </c>
+      <c r="B133" t="s">
+        <v>189</v>
+      </c>
+      <c r="C133" t="s">
+        <v>185</v>
+      </c>
+      <c r="D133">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>152</v>
+      </c>
+      <c r="B134" t="s">
+        <v>190</v>
+      </c>
+      <c r="C134" t="s">
+        <v>188</v>
+      </c>
+      <c r="D134">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>108</v>
+      </c>
+      <c r="B135" t="s">
+        <v>149</v>
+      </c>
+      <c r="C135" t="s">
+        <v>185</v>
+      </c>
+      <c r="D135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>109</v>
+      </c>
+      <c r="B136" t="s">
+        <v>190</v>
+      </c>
+      <c r="C136" t="s">
+        <v>188</v>
+      </c>
+      <c r="D136">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState ref="A2:E136">
+    <sortCondition ref="A1"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" t="s">
+        <v>146</v>
+      </c>
+      <c r="H3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add activity sleep and transformation systems
</commit_message>
<xml_diff>
--- a/assets_cropped/Tsurumaru Tsuyoshi/manifest_edit.xlsx
+++ b/assets_cropped/Tsurumaru Tsuyoshi/manifest_edit.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\TanukiProject\tanuki_app\assets_cropped\Tsurumaru Tsuyoshi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\TanukiProject\tanuki_app\assets_cropped\Tsurumaru Tsuyoshi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1776A0-449F-44BE-AD86-B9498FCCF5B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBCBDCF-618C-4717-AF59-9ACAB6BDD5B0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18510" windowHeight="5625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="209">
   <si>
     <t>filename</t>
   </si>
@@ -617,14 +617,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>window_walk,bottle_feed_child_approach,random</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>window_walk,bottle_feed_child_approach,negative_reaction,random</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>window_walk,random</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -666,6 +658,50 @@
   </si>
   <si>
     <t>window_walk,negative_reaction,random,bottle_feed_child_approach</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_denied,negative_reaction,random,activity_sleep_settling</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>random,activity_sleep_settling</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>activity_sleeping</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_denied,negative_reaction,random,activity_sleep_settling,activity_sleep_waking</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>random,activity_sleep_settling,activity_sleep_waking</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,random,activity_sleep_waking</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,negative_reaction,random,activity_sleep_waking,activity_sleep_observing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,random,activity_sleep_waking,activity_sleep_observing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,negative_reaction,random,activity_sleep_join_approach</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,bottle_feed_child_approach,negative_reaction,random,activity_sleep_join_approach</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,bottle_feed_child_approach,random,activity_sleep_join_approach</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1082,7 +1118,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C3" t="s">
         <v>161</v>
@@ -1096,7 +1132,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C4" t="s">
         <v>159</v>
@@ -1110,7 +1146,7 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C5" t="s">
         <v>162</v>
@@ -1124,7 +1160,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C6" t="s">
         <v>159</v>
@@ -1152,7 +1188,7 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C8" t="s">
         <v>159</v>
@@ -1166,7 +1202,7 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C9" t="s">
         <v>160</v>
@@ -1180,7 +1216,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C10" t="s">
         <v>163</v>
@@ -1194,7 +1230,7 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C11" t="s">
         <v>160</v>
@@ -1208,7 +1244,7 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C12" t="s">
         <v>173</v>
@@ -1236,7 +1272,7 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
@@ -1250,7 +1286,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C15" t="s">
         <v>154</v>
@@ -1278,7 +1314,7 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C17" t="s">
         <v>165</v>
@@ -1292,7 +1328,7 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C18" t="s">
         <v>158</v>
@@ -1306,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C19" t="s">
         <v>165</v>
@@ -1334,7 +1370,7 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C21" t="s">
         <v>158</v>
@@ -1348,10 +1384,10 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C22" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1362,7 +1398,7 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C23" t="s">
         <v>172</v>
@@ -1376,10 +1412,10 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C24" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1390,7 +1426,7 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C25" t="s">
         <v>176</v>
@@ -1407,7 +1443,7 @@
         <v>149</v>
       </c>
       <c r="C26" t="s">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1418,10 +1454,10 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C27" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1432,10 +1468,10 @@
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C28" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1460,7 +1496,7 @@
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C30" t="s">
         <v>6</v>
@@ -1488,7 +1524,7 @@
         <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C32" t="s">
         <v>154</v>
@@ -1502,7 +1538,7 @@
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C33" t="s">
         <v>6</v>
@@ -1516,7 +1552,7 @@
         <v>50</v>
       </c>
       <c r="B34" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C34" t="s">
         <v>177</v>
@@ -1530,7 +1566,7 @@
         <v>51</v>
       </c>
       <c r="B35" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C35" t="s">
         <v>177</v>
@@ -1544,7 +1580,7 @@
         <v>110</v>
       </c>
       <c r="B36" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C36" t="s">
         <v>178</v>
@@ -1558,7 +1594,7 @@
         <v>111</v>
       </c>
       <c r="B37" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C37" t="s">
         <v>179</v>
@@ -1572,7 +1608,7 @@
         <v>112</v>
       </c>
       <c r="B38" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C38" t="s">
         <v>178</v>
@@ -1600,7 +1636,7 @@
         <v>114</v>
       </c>
       <c r="B40" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C40" t="s">
         <v>179</v>
@@ -1628,10 +1664,10 @@
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C42" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1642,10 +1678,10 @@
         <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C43" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1656,10 +1692,10 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C44" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1684,7 +1720,7 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C46" t="s">
         <v>168</v>
@@ -1698,7 +1734,7 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C47" t="s">
         <v>157</v>
@@ -1712,7 +1748,7 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C48" t="s">
         <v>168</v>
@@ -1740,7 +1776,7 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C50" t="s">
         <v>157</v>
@@ -1754,7 +1790,7 @@
         <v>153</v>
       </c>
       <c r="B51" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C51" t="s">
         <v>181</v>
@@ -1782,7 +1818,7 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C53" t="s">
         <v>181</v>
@@ -1796,7 +1832,7 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C54" t="s">
         <v>178</v>
@@ -1810,7 +1846,7 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C55" t="s">
         <v>179</v>
@@ -1838,7 +1874,7 @@
         <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C57" t="s">
         <v>179</v>
@@ -1866,7 +1902,7 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C59" t="s">
         <v>168</v>
@@ -1880,7 +1916,7 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C60" t="s">
         <v>157</v>
@@ -1894,7 +1930,7 @@
         <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C61" t="s">
         <v>168</v>
@@ -1908,7 +1944,7 @@
         <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C62" t="s">
         <v>157</v>
@@ -1936,7 +1972,7 @@
         <v>73</v>
       </c>
       <c r="B64" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C64" t="s">
         <v>157</v>
@@ -1950,7 +1986,7 @@
         <v>78</v>
       </c>
       <c r="B65" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C65" t="s">
         <v>156</v>
@@ -1964,7 +2000,7 @@
         <v>79</v>
       </c>
       <c r="B66" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C66" t="s">
         <v>156</v>
@@ -1992,7 +2028,7 @@
         <v>75</v>
       </c>
       <c r="B68" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C68" t="s">
         <v>171</v>
@@ -2006,7 +2042,7 @@
         <v>76</v>
       </c>
       <c r="B69" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C69" t="s">
         <v>155</v>
@@ -2037,7 +2073,7 @@
         <v>149</v>
       </c>
       <c r="C71" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D71">
         <v>1</v>
@@ -2048,10 +2084,10 @@
         <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C72" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D72">
         <v>1</v>
@@ -2062,10 +2098,10 @@
         <v>82</v>
       </c>
       <c r="B73" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C73" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D73">
         <v>1</v>
@@ -2076,10 +2112,10 @@
         <v>83</v>
       </c>
       <c r="B74" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C74" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D74">
         <v>1</v>
@@ -2093,7 +2129,7 @@
         <v>149</v>
       </c>
       <c r="C75" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D75">
         <v>1</v>
@@ -2104,10 +2140,10 @@
         <v>85</v>
       </c>
       <c r="B76" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C76" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D76">
         <v>1</v>
@@ -2132,7 +2168,7 @@
         <v>117</v>
       </c>
       <c r="B78" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C78" t="s">
         <v>154</v>
@@ -2160,7 +2196,7 @@
         <v>40</v>
       </c>
       <c r="B80" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C80" t="s">
         <v>183</v>
@@ -2174,7 +2210,7 @@
         <v>41</v>
       </c>
       <c r="B81" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C81" t="s">
         <v>177</v>
@@ -2188,7 +2224,7 @@
         <v>42</v>
       </c>
       <c r="B82" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C82" t="s">
         <v>183</v>
@@ -2216,7 +2252,7 @@
         <v>44</v>
       </c>
       <c r="B84" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C84" t="s">
         <v>183</v>
@@ -2230,7 +2266,7 @@
         <v>45</v>
       </c>
       <c r="B85" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C85" t="s">
         <v>154</v>
@@ -2244,7 +2280,7 @@
         <v>46</v>
       </c>
       <c r="B86" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C86" t="s">
         <v>177</v>
@@ -2258,7 +2294,7 @@
         <v>47</v>
       </c>
       <c r="B87" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C87" t="s">
         <v>154</v>
@@ -2286,7 +2322,7 @@
         <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C89" t="s">
         <v>175</v>
@@ -2300,7 +2336,7 @@
         <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C90" t="s">
         <v>173</v>
@@ -2314,7 +2350,7 @@
         <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C91" t="s">
         <v>175</v>
@@ -2342,7 +2378,7 @@
         <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C93" t="s">
         <v>173</v>
@@ -2356,10 +2392,10 @@
         <v>118</v>
       </c>
       <c r="B94" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C94" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D94">
         <v>1</v>
@@ -2373,7 +2409,7 @@
         <v>149</v>
       </c>
       <c r="C95" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -2384,10 +2420,10 @@
         <v>120</v>
       </c>
       <c r="B96" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C96" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D96">
         <v>1</v>
@@ -2401,7 +2437,7 @@
         <v>149</v>
       </c>
       <c r="C97" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D97">
         <v>1</v>
@@ -2412,10 +2448,10 @@
         <v>122</v>
       </c>
       <c r="B98" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C98" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D98">
         <v>1</v>
@@ -2426,10 +2462,10 @@
         <v>123</v>
       </c>
       <c r="B99" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C99" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D99">
         <v>1</v>
@@ -2440,10 +2476,10 @@
         <v>124</v>
       </c>
       <c r="B100" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C100" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D100">
         <v>1</v>
@@ -2482,7 +2518,7 @@
         <v>127</v>
       </c>
       <c r="B103" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C103" t="s">
         <v>174</v>
@@ -2496,7 +2532,7 @@
         <v>128</v>
       </c>
       <c r="B104" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C104" t="s">
         <v>173</v>
@@ -2510,7 +2546,7 @@
         <v>129</v>
       </c>
       <c r="B105" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C105" t="s">
         <v>174</v>
@@ -2524,7 +2560,7 @@
         <v>130</v>
       </c>
       <c r="B106" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C106" t="s">
         <v>173</v>
@@ -2566,7 +2602,7 @@
         <v>133</v>
       </c>
       <c r="B109" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C109" t="s">
         <v>173</v>
@@ -2594,7 +2630,7 @@
         <v>135</v>
       </c>
       <c r="B111" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C111" t="s">
         <v>182</v>
@@ -2608,7 +2644,7 @@
         <v>136</v>
       </c>
       <c r="B112" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C112" t="s">
         <v>181</v>
@@ -2650,7 +2686,7 @@
         <v>139</v>
       </c>
       <c r="B115" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C115" t="s">
         <v>181</v>
@@ -2678,10 +2714,10 @@
         <v>93</v>
       </c>
       <c r="B117" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C117" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -2692,10 +2728,10 @@
         <v>94</v>
       </c>
       <c r="B118" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C118" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -2706,7 +2742,7 @@
         <v>95</v>
       </c>
       <c r="B119" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C119" t="s">
         <v>182</v>
@@ -2723,7 +2759,7 @@
         <v>149</v>
       </c>
       <c r="C120" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -2734,10 +2770,10 @@
         <v>97</v>
       </c>
       <c r="B121" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C121" t="s">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -2748,7 +2784,7 @@
         <v>98</v>
       </c>
       <c r="B122" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C122" t="s">
         <v>181</v>
@@ -2790,10 +2826,10 @@
         <v>101</v>
       </c>
       <c r="B125" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C125" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -2804,10 +2840,10 @@
         <v>102</v>
       </c>
       <c r="B126" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C126" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -2818,10 +2854,10 @@
         <v>103</v>
       </c>
       <c r="B127" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C127" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -2835,7 +2871,7 @@
         <v>149</v>
       </c>
       <c r="C128" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -2846,10 +2882,10 @@
         <v>105</v>
       </c>
       <c r="B129" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C129" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -2874,7 +2910,7 @@
         <v>150</v>
       </c>
       <c r="B131" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C131" t="s">
         <v>185</v>
@@ -2888,10 +2924,10 @@
         <v>107</v>
       </c>
       <c r="B132" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C132" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -2902,7 +2938,7 @@
         <v>151</v>
       </c>
       <c r="B133" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C133" t="s">
         <v>185</v>
@@ -2916,10 +2952,10 @@
         <v>152</v>
       </c>
       <c r="B134" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C134" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -2944,10 +2980,10 @@
         <v>109</v>
       </c>
       <c r="B136" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C136" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D136">
         <v>1</v>

</xml_diff>